<commit_message>
fixed half of the excel file for the ai
</commit_message>
<xml_diff>
--- a/ML Progress Sheet.xlsx
+++ b/ML Progress Sheet.xlsx
@@ -2739,7 +2739,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2784,18 +2784,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor rgb="FFFEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF967656"/>
-        <bgColor rgb="FF9C6500"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFF1F5F9"/>
       </patternFill>
@@ -2809,6 +2797,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFEE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor rgb="FFFEE2E2"/>
       </patternFill>
     </fill>
@@ -2880,172 +2874,160 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3133,14 +3115,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FF006100"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -3181,6 +3155,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -3204,7 +3186,7 @@
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFCCCCCC"/>
-      <rgbColor rgb="FF967656"/>
+      <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF1F5F9"/>
@@ -4342,7 +4324,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="44" s="15" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" s="14" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
         <v>164</v>
       </c>
@@ -4365,7 +4347,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="45" s="15" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" s="14" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
         <v>168</v>
       </c>
@@ -4445,7 +4427,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="49" s="15" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" s="14" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="10" t="s">
         <v>181</v>
       </c>
@@ -4468,7 +4450,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" s="16" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" s="9" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>185</v>
       </c>
@@ -4697,7 +4679,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="61" s="16" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" s="9" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
         <v>224</v>
       </c>
@@ -4743,60 +4725,60 @@
         <v>232</v>
       </c>
     </row>
-    <row r="63" s="18" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="17" t="s">
+    <row r="63" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="B63" s="17"/>
-      <c r="C63" s="17"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="17"/>
-      <c r="G63" s="17"/>
-    </row>
-    <row r="64" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="19" t="s">
+      <c r="B63" s="15"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="15"/>
+      <c r="G63" s="15"/>
+    </row>
+    <row r="64" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="B64" s="20" t="s">
+      <c r="B64" s="17" t="s">
         <v>235</v>
       </c>
-      <c r="C64" s="21" t="s">
+      <c r="C64" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D64" s="22" t="s">
+      <c r="D64" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E64" s="20" t="s">
+      <c r="E64" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F64" s="20" t="s">
+      <c r="F64" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="G64" s="20" t="s">
+      <c r="G64" s="17" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="65" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="19" t="s">
+    <row r="65" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="16" t="s">
         <v>240</v>
       </c>
-      <c r="B65" s="20" t="s">
+      <c r="B65" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="C65" s="21" t="s">
+      <c r="C65" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D65" s="22" t="s">
+      <c r="D65" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E65" s="20" t="s">
+      <c r="E65" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F65" s="20" t="s">
+      <c r="F65" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="G65" s="20" t="s">
+      <c r="G65" s="17" t="s">
         <v>243</v>
       </c>
     </row>
@@ -4961,26 +4943,26 @@
         <v>274</v>
       </c>
     </row>
-    <row r="73" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="19" t="s">
+    <row r="73" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A73" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="B73" s="20" t="s">
+      <c r="B73" s="17" t="s">
         <v>276</v>
       </c>
-      <c r="C73" s="24" t="s">
+      <c r="C73" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D73" s="25" t="s">
+      <c r="D73" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E73" s="20" t="s">
+      <c r="E73" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F73" s="20" t="s">
+      <c r="F73" s="17" t="s">
         <v>277</v>
       </c>
-      <c r="G73" s="20" t="s">
+      <c r="G73" s="17" t="s">
         <v>278</v>
       </c>
     </row>
@@ -5007,49 +4989,49 @@
         <v>282</v>
       </c>
     </row>
-    <row r="75" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="19" t="s">
+    <row r="75" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="16" t="s">
         <v>283</v>
       </c>
-      <c r="B75" s="20" t="s">
+      <c r="B75" s="17" t="s">
         <v>284</v>
       </c>
-      <c r="C75" s="24" t="s">
+      <c r="C75" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D75" s="25" t="s">
+      <c r="D75" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E75" s="20" t="s">
+      <c r="E75" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F75" s="20" t="s">
+      <c r="F75" s="17" t="s">
         <v>285</v>
       </c>
-      <c r="G75" s="20" t="s">
+      <c r="G75" s="17" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="76" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="19" t="s">
+    <row r="76" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="16" t="s">
         <v>287</v>
       </c>
-      <c r="B76" s="20" t="s">
+      <c r="B76" s="17" t="s">
         <v>288</v>
       </c>
-      <c r="C76" s="24" t="s">
+      <c r="C76" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D76" s="25" t="s">
+      <c r="D76" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E76" s="20" t="s">
+      <c r="E76" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F76" s="20" t="s">
+      <c r="F76" s="17" t="s">
         <v>289</v>
       </c>
-      <c r="G76" s="20" t="s">
+      <c r="G76" s="17" t="s">
         <v>290</v>
       </c>
     </row>
@@ -5076,37 +5058,37 @@
         <v>294</v>
       </c>
     </row>
-    <row r="78" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="26" t="s">
+    <row r="78" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="B78" s="26"/>
-      <c r="C78" s="26"/>
-      <c r="D78" s="26"/>
-      <c r="E78" s="26"/>
-      <c r="F78" s="26"/>
-      <c r="G78" s="26"/>
-    </row>
-    <row r="79" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="19" t="s">
+      <c r="B78" s="21"/>
+      <c r="C78" s="21"/>
+      <c r="D78" s="21"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="21"/>
+      <c r="G78" s="21"/>
+    </row>
+    <row r="79" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="B79" s="20" t="s">
+      <c r="B79" s="17" t="s">
         <v>297</v>
       </c>
-      <c r="C79" s="24" t="s">
+      <c r="C79" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D79" s="25" t="s">
+      <c r="D79" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E79" s="20" t="s">
+      <c r="E79" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F79" s="20" t="s">
+      <c r="F79" s="17" t="s">
         <v>298</v>
       </c>
-      <c r="G79" s="20" t="s">
+      <c r="G79" s="17" t="s">
         <v>299</v>
       </c>
     </row>
@@ -5133,49 +5115,49 @@
         <v>303</v>
       </c>
     </row>
-    <row r="81" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="19" t="s">
+    <row r="81" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="B81" s="20" t="s">
+      <c r="B81" s="17" t="s">
         <v>305</v>
       </c>
-      <c r="C81" s="24" t="s">
+      <c r="C81" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D81" s="25" t="s">
+      <c r="D81" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E81" s="20" t="s">
+      <c r="E81" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F81" s="20" t="s">
+      <c r="F81" s="17" t="s">
         <v>306</v>
       </c>
-      <c r="G81" s="20" t="s">
+      <c r="G81" s="17" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="82" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A82" s="19" t="s">
+    <row r="82" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="16" t="s">
         <v>308</v>
       </c>
-      <c r="B82" s="20" t="s">
+      <c r="B82" s="17" t="s">
         <v>309</v>
       </c>
-      <c r="C82" s="24" t="s">
+      <c r="C82" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D82" s="25" t="s">
+      <c r="D82" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E82" s="20" t="s">
+      <c r="E82" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F82" s="20" t="s">
+      <c r="F82" s="17" t="s">
         <v>310</v>
       </c>
-      <c r="G82" s="20" t="s">
+      <c r="G82" s="17" t="s">
         <v>311</v>
       </c>
     </row>
@@ -5225,26 +5207,26 @@
         <v>319</v>
       </c>
     </row>
-    <row r="85" s="23" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A85" s="19" t="s">
+    <row r="85" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A85" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="B85" s="20" t="s">
+      <c r="B85" s="17" t="s">
         <v>321</v>
       </c>
-      <c r="C85" s="24" t="s">
+      <c r="C85" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="D85" s="25" t="s">
+      <c r="D85" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="E85" s="20" t="s">
+      <c r="E85" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="F85" s="20" t="s">
+      <c r="F85" s="17" t="s">
         <v>322</v>
       </c>
-      <c r="G85" s="20" t="s">
+      <c r="G85" s="17" t="s">
         <v>323</v>
       </c>
     </row>
@@ -5295,10 +5277,10 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B88" s="23"/>
+      <c r="B88" s="22"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C89" s="27"/>
+      <c r="C89" s="22"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:G87"/>
@@ -5381,206 +5363,206 @@
       <c r="E4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="23" t="s">
         <v>336</v>
       </c>
-      <c r="B5" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="30" t="s">
+      <c r="B5" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="31" t="s">
+      <c r="D5" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="26" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="23" t="s">
         <v>337</v>
       </c>
-      <c r="B6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="30" t="s">
+      <c r="B6" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="26" t="s">
         <v>338</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="26" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="23" t="s">
         <v>339</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="D7" s="31" t="s">
+      <c r="D7" s="26" t="s">
         <v>340</v>
       </c>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="26" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="23" t="s">
         <v>342</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D8" s="26" t="s">
         <v>343</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="26" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="23" t="s">
         <v>345</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="D9" s="31" t="s">
+      <c r="D9" s="26" t="s">
         <v>346</v>
       </c>
-      <c r="E9" s="31" t="s">
+      <c r="E9" s="26" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="23" t="s">
         <v>348</v>
       </c>
-      <c r="B10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="30" t="s">
+      <c r="B10" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="26" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="23" t="s">
         <v>350</v>
       </c>
-      <c r="B11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="30" t="s">
+      <c r="B11" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="26" t="s">
         <v>351</v>
       </c>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="26" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="23" t="s">
         <v>353</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="26" t="s">
         <v>354</v>
       </c>
-      <c r="E12" s="31" t="s">
+      <c r="E12" s="26" t="s">
         <v>355</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="23" t="s">
         <v>356</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="26" t="s">
         <v>357</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="E13" s="26" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>359</v>
       </c>
-      <c r="B14" s="32" t="s">
+      <c r="B14" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="26" t="s">
         <v>360</v>
       </c>
-      <c r="E14" s="31" t="s">
+      <c r="E14" s="26" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="23" t="s">
         <v>361</v>
       </c>
-      <c r="B15" s="32" t="s">
+      <c r="B15" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="28" t="s">
         <v>230</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="26" t="s">
         <v>231</v>
       </c>
-      <c r="E15" s="31" t="s">
+      <c r="E15" s="26" t="s">
         <v>362</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="23" t="s">
         <v>363</v>
       </c>
-      <c r="B16" s="32" t="s">
+      <c r="B16" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="E16" s="31" t="s">
+      <c r="E16" s="26" t="s">
         <v>364</v>
       </c>
     </row>
@@ -5594,104 +5576,104 @@
       <c r="E17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="23" t="s">
         <v>366</v>
       </c>
-      <c r="B18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C18" s="30" t="s">
+      <c r="B18" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D18" s="31" t="s">
+      <c r="D18" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="31" t="s">
+      <c r="E18" s="26" t="s">
         <v>367</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="23" t="s">
         <v>368</v>
       </c>
-      <c r="B19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C19" s="30" t="s">
+      <c r="B19" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D19" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="E19" s="31" t="s">
+      <c r="E19" s="26" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="23" t="s">
         <v>370</v>
       </c>
-      <c r="B20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C20" s="30" t="s">
+      <c r="B20" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="31" t="s">
+      <c r="D20" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="31" t="s">
+      <c r="E20" s="26" t="s">
         <v>371</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="23" t="s">
         <v>372</v>
       </c>
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D21" s="31" t="s">
+      <c r="D21" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="E21" s="31" t="s">
+      <c r="E21" s="26" t="s">
         <v>373</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="23" t="s">
         <v>374</v>
       </c>
-      <c r="B22" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="30" t="s">
+      <c r="B22" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D22" s="31" t="s">
+      <c r="D22" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="E22" s="31" t="s">
+      <c r="E22" s="26" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="23" t="s">
         <v>376</v>
       </c>
-      <c r="B23" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="30" t="s">
+      <c r="B23" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="31" t="s">
+      <c r="D23" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="31" t="s">
+      <c r="E23" s="26" t="s">
         <v>377</v>
       </c>
     </row>
@@ -5705,70 +5687,70 @@
       <c r="E24" s="4"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>379</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="31" t="s">
+      <c r="D25" s="26" t="s">
         <v>380</v>
       </c>
-      <c r="E25" s="31" t="s">
+      <c r="E25" s="26" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="23" t="s">
         <v>382</v>
       </c>
-      <c r="B26" s="32" t="s">
+      <c r="B26" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="33" t="s">
+      <c r="C26" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="31" t="s">
+      <c r="D26" s="26" t="s">
         <v>383</v>
       </c>
-      <c r="E26" s="31" t="s">
+      <c r="E26" s="26" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="23" t="s">
         <v>385</v>
       </c>
-      <c r="B27" s="32" t="s">
+      <c r="B27" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="D27" s="31" t="s">
+      <c r="D27" s="26" t="s">
         <v>386</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="26" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="23" t="s">
         <v>388</v>
       </c>
-      <c r="B28" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="30" t="s">
+      <c r="B28" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="31" t="s">
+      <c r="D28" s="26" t="s">
         <v>389</v>
       </c>
-      <c r="E28" s="31" t="s">
+      <c r="E28" s="26" t="s">
         <v>390</v>
       </c>
     </row>
@@ -5782,223 +5764,223 @@
       <c r="E29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="23" t="s">
         <v>392</v>
       </c>
-      <c r="B30" s="24" t="s">
+      <c r="B30" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C30" s="25" t="s">
+      <c r="C30" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="D30" s="26" t="s">
         <v>393</v>
       </c>
-      <c r="E30" s="31" t="s">
+      <c r="E30" s="26" t="s">
         <v>394</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="23" t="s">
         <v>395</v>
       </c>
-      <c r="B31" s="24" t="s">
+      <c r="B31" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C31" s="25" t="s">
+      <c r="C31" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D31" s="31" t="s">
+      <c r="D31" s="26" t="s">
         <v>242</v>
       </c>
-      <c r="E31" s="31" t="s">
+      <c r="E31" s="26" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="23" t="s">
         <v>397</v>
       </c>
-      <c r="B32" s="32" t="s">
+      <c r="B32" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C32" s="33" t="s">
+      <c r="C32" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="D32" s="31" t="s">
+      <c r="D32" s="26" t="s">
         <v>398</v>
       </c>
-      <c r="E32" s="31" t="s">
+      <c r="E32" s="26" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28" t="s">
+      <c r="A33" s="23" t="s">
         <v>400</v>
       </c>
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="33" t="s">
+      <c r="C33" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="D33" s="31" t="s">
+      <c r="D33" s="26" t="s">
         <v>255</v>
       </c>
-      <c r="E33" s="31" t="s">
+      <c r="E33" s="26" t="s">
         <v>401</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
+      <c r="A34" s="23" t="s">
         <v>402</v>
       </c>
-      <c r="B34" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="C34" s="30" t="s">
+      <c r="B34" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C34" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="D34" s="31" t="s">
+      <c r="D34" s="26" t="s">
         <v>403</v>
       </c>
-      <c r="E34" s="31" t="s">
+      <c r="E34" s="26" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="23" t="s">
         <v>405</v>
       </c>
-      <c r="B35" s="32" t="s">
+      <c r="B35" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C35" s="33" t="s">
+      <c r="C35" s="28" t="s">
         <v>263</v>
       </c>
-      <c r="D35" s="31" t="s">
+      <c r="D35" s="26" t="s">
         <v>406</v>
       </c>
-      <c r="E35" s="31" t="s">
+      <c r="E35" s="26" t="s">
         <v>407</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="23" t="s">
         <v>408</v>
       </c>
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C36" s="33" t="s">
+      <c r="C36" s="28" t="s">
         <v>268</v>
       </c>
-      <c r="D36" s="31" t="s">
+      <c r="D36" s="26" t="s">
         <v>409</v>
       </c>
-      <c r="E36" s="31" t="s">
+      <c r="E36" s="26" t="s">
         <v>410</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="23" t="s">
         <v>411</v>
       </c>
-      <c r="B37" s="32" t="s">
+      <c r="B37" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C37" s="33" t="s">
+      <c r="C37" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="D37" s="31" t="s">
+      <c r="D37" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="E37" s="31" t="s">
+      <c r="E37" s="26" t="s">
         <v>412</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="23" t="s">
         <v>413</v>
       </c>
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C38" s="25" t="s">
+      <c r="C38" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D38" s="31" t="s">
+      <c r="D38" s="26" t="s">
         <v>414</v>
       </c>
-      <c r="E38" s="31" t="s">
+      <c r="E38" s="26" t="s">
         <v>278</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="28" t="s">
+      <c r="A39" s="23" t="s">
         <v>415</v>
       </c>
-      <c r="B39" s="32" t="s">
+      <c r="B39" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C39" s="33" t="s">
+      <c r="C39" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="D39" s="31" t="s">
+      <c r="D39" s="26" t="s">
         <v>416</v>
       </c>
-      <c r="E39" s="31" t="s">
+      <c r="E39" s="26" t="s">
         <v>417</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="s">
+      <c r="A40" s="23" t="s">
         <v>418</v>
       </c>
-      <c r="B40" s="24" t="s">
+      <c r="B40" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D40" s="31" t="s">
+      <c r="D40" s="26" t="s">
         <v>419</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="26" t="s">
         <v>286</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="23" t="s">
         <v>420</v>
       </c>
-      <c r="B41" s="24" t="s">
+      <c r="B41" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C41" s="25" t="s">
+      <c r="C41" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D41" s="31" t="s">
+      <c r="D41" s="26" t="s">
         <v>421</v>
       </c>
-      <c r="E41" s="31" t="s">
+      <c r="E41" s="26" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="s">
+      <c r="A42" s="23" t="s">
         <v>423</v>
       </c>
-      <c r="B42" s="32" t="s">
+      <c r="B42" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C42" s="33" t="s">
+      <c r="C42" s="28" t="s">
         <v>268</v>
       </c>
-      <c r="D42" s="31" t="s">
+      <c r="D42" s="26" t="s">
         <v>293</v>
       </c>
-      <c r="E42" s="31" t="s">
+      <c r="E42" s="26" t="s">
         <v>424</v>
       </c>
     </row>
@@ -6012,121 +5994,121 @@
       <c r="E43" s="4"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="28" t="s">
+      <c r="A44" s="23" t="s">
         <v>426</v>
       </c>
-      <c r="B44" s="24" t="s">
+      <c r="B44" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C44" s="25" t="s">
+      <c r="C44" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D44" s="31" t="s">
+      <c r="D44" s="26" t="s">
         <v>427</v>
       </c>
-      <c r="E44" s="31" t="s">
+      <c r="E44" s="26" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="23" t="s">
         <v>429</v>
       </c>
-      <c r="B45" s="32" t="s">
+      <c r="B45" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C45" s="33" t="s">
+      <c r="C45" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="D45" s="31" t="s">
+      <c r="D45" s="26" t="s">
         <v>430</v>
       </c>
-      <c r="E45" s="31" t="s">
+      <c r="E45" s="26" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="28" t="s">
+      <c r="A46" s="23" t="s">
         <v>432</v>
       </c>
-      <c r="B46" s="24" t="s">
+      <c r="B46" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C46" s="25" t="s">
+      <c r="C46" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D46" s="31" t="s">
+      <c r="D46" s="26" t="s">
         <v>306</v>
       </c>
-      <c r="E46" s="31" t="s">
+      <c r="E46" s="26" t="s">
         <v>307</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="23" t="s">
         <v>433</v>
       </c>
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C47" s="25" t="s">
+      <c r="C47" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D47" s="31" t="s">
+      <c r="D47" s="26" t="s">
         <v>434</v>
       </c>
-      <c r="E47" s="31" t="s">
+      <c r="E47" s="26" t="s">
         <v>311</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28" t="s">
+      <c r="A48" s="23" t="s">
         <v>435</v>
       </c>
-      <c r="B48" s="32" t="s">
+      <c r="B48" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C48" s="33" t="s">
+      <c r="C48" s="28" t="s">
         <v>230</v>
       </c>
-      <c r="D48" s="31" t="s">
+      <c r="D48" s="26" t="s">
         <v>436</v>
       </c>
-      <c r="E48" s="31" t="s">
+      <c r="E48" s="26" t="s">
         <v>437</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="23" t="s">
         <v>438</v>
       </c>
-      <c r="B49" s="32" t="s">
+      <c r="B49" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="33" t="s">
+      <c r="C49" s="28" t="s">
         <v>254</v>
       </c>
-      <c r="D49" s="31" t="s">
+      <c r="D49" s="26" t="s">
         <v>439</v>
       </c>
-      <c r="E49" s="31" t="s">
+      <c r="E49" s="26" t="s">
         <v>440</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="28" t="s">
+      <c r="A50" s="23" t="s">
         <v>441</v>
       </c>
-      <c r="B50" s="24" t="s">
+      <c r="B50" s="29" t="s">
         <v>236</v>
       </c>
-      <c r="C50" s="25" t="s">
+      <c r="C50" s="30" t="s">
         <v>237</v>
       </c>
-      <c r="D50" s="31" t="s">
+      <c r="D50" s="26" t="s">
         <v>322</v>
       </c>
-      <c r="E50" s="31" t="s">
+      <c r="E50" s="26" t="s">
         <v>442</v>
       </c>
     </row>
@@ -6210,142 +6192,142 @@
       <c r="F4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="23" t="s">
         <v>449</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="26" t="s">
         <v>450</v>
       </c>
-      <c r="C5" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="30" t="s">
+      <c r="C5" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E5" s="31" t="s">
+      <c r="E5" s="26" t="s">
         <v>452</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="26" t="s">
         <v>453</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="23" t="s">
         <v>454</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="26" t="s">
         <v>455</v>
       </c>
-      <c r="C6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="30" t="s">
+      <c r="C6" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="26" t="s">
         <v>456</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="26" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="23" t="s">
         <v>458</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="26" t="s">
         <v>459</v>
       </c>
-      <c r="C7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="30" t="s">
+      <c r="C7" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="26" t="s">
         <v>460</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="26" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="23" t="s">
         <v>461</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="26" t="s">
         <v>462</v>
       </c>
-      <c r="C8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="30" t="s">
+      <c r="C8" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="26" t="s">
         <v>463</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="26" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="23" t="s">
         <v>464</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="26" t="s">
         <v>465</v>
       </c>
-      <c r="C9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="30" t="s">
+      <c r="C9" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E9" s="31" t="s">
+      <c r="E9" s="26" t="s">
         <v>466</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="26" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="23" t="s">
         <v>467</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="26" t="s">
         <v>468</v>
       </c>
-      <c r="C10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="30" t="s">
+      <c r="C10" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E10" s="31" t="s">
+      <c r="E10" s="26" t="s">
         <v>469</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="26" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="23" t="s">
         <v>470</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="26" t="s">
         <v>471</v>
       </c>
-      <c r="C11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="30" t="s">
+      <c r="C11" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E11" s="31" t="s">
+      <c r="E11" s="26" t="s">
         <v>472</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="26" t="s">
         <v>473</v>
       </c>
     </row>
@@ -6360,262 +6342,262 @@
       <c r="F12" s="4"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="23" t="s">
         <v>475</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="26" t="s">
         <v>476</v>
       </c>
-      <c r="C13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="30" t="s">
+      <c r="C13" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E13" s="31" t="s">
+      <c r="E13" s="26" t="s">
         <v>477</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="26" t="s">
         <v>478</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>479</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="26" t="s">
         <v>480</v>
       </c>
-      <c r="C14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="30" t="s">
+      <c r="C14" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E14" s="31" t="s">
+      <c r="E14" s="26" t="s">
         <v>481</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="23" t="s">
         <v>483</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="26" t="s">
         <v>484</v>
       </c>
-      <c r="C15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E15" s="31" t="s">
+      <c r="E15" s="26" t="s">
         <v>485</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="23" t="s">
         <v>486</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="26" t="s">
         <v>487</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E16" s="31" t="s">
+      <c r="E16" s="26" t="s">
         <v>485</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="23" t="s">
         <v>488</v>
       </c>
-      <c r="B17" s="31" t="s">
+      <c r="B17" s="26" t="s">
         <v>489</v>
       </c>
-      <c r="C17" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E17" s="31" t="s">
+      <c r="E17" s="26" t="s">
         <v>485</v>
       </c>
-      <c r="F17" s="31" t="s">
+      <c r="F17" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="23" t="s">
         <v>490</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="26" t="s">
         <v>491</v>
       </c>
-      <c r="C18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E18" s="31" t="s">
+      <c r="E18" s="26" t="s">
         <v>492</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="23" t="s">
         <v>493</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="26" t="s">
         <v>494</v>
       </c>
-      <c r="C19" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E19" s="31" t="s">
+      <c r="E19" s="26" t="s">
         <v>495</v>
       </c>
-      <c r="F19" s="31" t="s">
+      <c r="F19" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="23" t="s">
         <v>496</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="26" t="s">
         <v>497</v>
       </c>
-      <c r="C20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="30" t="s">
+      <c r="C20" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E20" s="31" t="s">
+      <c r="E20" s="26" t="s">
         <v>498</v>
       </c>
-      <c r="F20" s="31" t="s">
+      <c r="F20" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="23" t="s">
         <v>499</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="26" t="s">
         <v>500</v>
       </c>
-      <c r="C21" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E21" s="31" t="s">
+      <c r="E21" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F21" s="31" t="s">
+      <c r="F21" s="26" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="26" t="s">
         <v>504</v>
       </c>
-      <c r="C22" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="30" t="s">
+      <c r="C22" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E22" s="31" t="s">
+      <c r="E22" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F22" s="31" t="s">
+      <c r="F22" s="26" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="23" t="s">
         <v>505</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="26" t="s">
         <v>506</v>
       </c>
-      <c r="C23" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="30" t="s">
+      <c r="C23" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E23" s="31" t="s">
+      <c r="E23" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F23" s="31" t="s">
+      <c r="F23" s="26" t="s">
         <v>502</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="23" t="s">
         <v>507</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="26" t="s">
         <v>508</v>
       </c>
-      <c r="C24" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="30" t="s">
+      <c r="C24" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E24" s="31" t="s">
+      <c r="E24" s="26" t="s">
         <v>509</v>
       </c>
-      <c r="F24" s="31" t="s">
+      <c r="F24" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>510</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="26" t="s">
         <v>511</v>
       </c>
-      <c r="C25" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="30" t="s">
+      <c r="C25" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E25" s="31" t="s">
+      <c r="E25" s="26" t="s">
         <v>512</v>
       </c>
-      <c r="F25" s="31" t="s">
+      <c r="F25" s="26" t="s">
         <v>482</v>
       </c>
     </row>
@@ -6630,242 +6612,242 @@
       <c r="F26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="23" t="s">
         <v>514</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="26" t="s">
         <v>515</v>
       </c>
-      <c r="C27" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="30" t="s">
+      <c r="C27" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E27" s="31" t="s">
+      <c r="E27" s="26" t="s">
         <v>516</v>
       </c>
-      <c r="F27" s="31" t="s">
+      <c r="F27" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="23" t="s">
         <v>517</v>
       </c>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="26" t="s">
         <v>518</v>
       </c>
-      <c r="C28" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="30" t="s">
+      <c r="C28" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E28" s="31" t="s">
+      <c r="E28" s="26" t="s">
         <v>519</v>
       </c>
-      <c r="F28" s="31" t="s">
+      <c r="F28" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="28" t="s">
+      <c r="A29" s="23" t="s">
         <v>520</v>
       </c>
-      <c r="B29" s="31" t="s">
+      <c r="B29" s="26" t="s">
         <v>521</v>
       </c>
-      <c r="C29" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="30" t="s">
+      <c r="C29" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E29" s="31" t="s">
+      <c r="E29" s="26" t="s">
         <v>519</v>
       </c>
-      <c r="F29" s="31" t="s">
+      <c r="F29" s="26" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="28" t="s">
+      <c r="A30" s="23" t="s">
         <v>523</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="26" t="s">
         <v>524</v>
       </c>
-      <c r="C30" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="30" t="s">
+      <c r="C30" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E30" s="31" t="s">
+      <c r="E30" s="26" t="s">
         <v>519</v>
       </c>
-      <c r="F30" s="31" t="s">
+      <c r="F30" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="28" t="s">
+      <c r="A31" s="23" t="s">
         <v>525</v>
       </c>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="26" t="s">
         <v>526</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="E31" s="31" t="s">
+      <c r="E31" s="26" t="s">
         <v>519</v>
       </c>
-      <c r="F31" s="31" t="s">
+      <c r="F31" s="26" t="s">
         <v>527</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
+      <c r="A32" s="23" t="s">
         <v>528</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="26" t="s">
         <v>529</v>
       </c>
-      <c r="C32" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="30" t="s">
+      <c r="C32" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E32" s="31" t="s">
+      <c r="E32" s="26" t="s">
         <v>519</v>
       </c>
-      <c r="F32" s="31" t="s">
+      <c r="F32" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="28" t="s">
+      <c r="A33" s="23" t="s">
         <v>530</v>
       </c>
-      <c r="B33" s="31" t="s">
+      <c r="B33" s="26" t="s">
         <v>531</v>
       </c>
-      <c r="C33" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="30" t="s">
+      <c r="C33" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E33" s="31" t="s">
+      <c r="E33" s="26" t="s">
         <v>532</v>
       </c>
-      <c r="F33" s="31" t="s">
+      <c r="F33" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="28" t="s">
+      <c r="A34" s="23" t="s">
         <v>533</v>
       </c>
-      <c r="B34" s="31" t="s">
+      <c r="B34" s="26" t="s">
         <v>534</v>
       </c>
-      <c r="C34" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="30" t="s">
+      <c r="C34" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E34" s="31" t="s">
+      <c r="E34" s="26" t="s">
         <v>532</v>
       </c>
-      <c r="F34" s="31" t="s">
+      <c r="F34" s="26" t="s">
         <v>535</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="23" t="s">
         <v>536</v>
       </c>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="26" t="s">
         <v>537</v>
       </c>
-      <c r="C35" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="30" t="s">
+      <c r="C35" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E35" s="31" t="s">
+      <c r="E35" s="26" t="s">
         <v>538</v>
       </c>
-      <c r="F35" s="31" t="s">
+      <c r="F35" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="28" t="s">
+      <c r="A36" s="23" t="s">
         <v>539</v>
       </c>
-      <c r="B36" s="31" t="s">
+      <c r="B36" s="26" t="s">
         <v>540</v>
       </c>
-      <c r="C36" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="30" t="s">
+      <c r="C36" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E36" s="31" t="s">
+      <c r="E36" s="26" t="s">
         <v>541</v>
       </c>
-      <c r="F36" s="31" t="s">
+      <c r="F36" s="26" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="28" t="s">
+      <c r="A37" s="23" t="s">
         <v>543</v>
       </c>
-      <c r="B37" s="31" t="s">
+      <c r="B37" s="26" t="s">
         <v>544</v>
       </c>
-      <c r="C37" s="32" t="s">
+      <c r="C37" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D37" s="33" t="s">
+      <c r="D37" s="28" t="s">
         <v>206</v>
       </c>
-      <c r="E37" s="31" t="s">
+      <c r="E37" s="26" t="s">
         <v>545</v>
       </c>
-      <c r="F37" s="31" t="s">
+      <c r="F37" s="26" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="23" t="s">
         <v>547</v>
       </c>
-      <c r="B38" s="31" t="s">
+      <c r="B38" s="26" t="s">
         <v>548</v>
       </c>
-      <c r="C38" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="30" t="s">
+      <c r="C38" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E38" s="31" t="s">
+      <c r="E38" s="26" t="s">
         <v>549</v>
       </c>
-      <c r="F38" s="31" t="s">
+      <c r="F38" s="26" t="s">
         <v>482</v>
       </c>
     </row>
@@ -6880,422 +6862,422 @@
       <c r="F39" s="4"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="28" t="s">
+      <c r="A40" s="23" t="s">
         <v>551</v>
       </c>
-      <c r="B40" s="31" t="s">
+      <c r="B40" s="26" t="s">
         <v>552</v>
       </c>
-      <c r="C40" s="32" t="s">
+      <c r="C40" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D40" s="33" t="s">
+      <c r="D40" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="E40" s="31" t="s">
+      <c r="E40" s="26" t="s">
         <v>553</v>
       </c>
-      <c r="F40" s="31" t="s">
+      <c r="F40" s="26" t="s">
         <v>554</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="28" t="s">
+      <c r="A41" s="23" t="s">
         <v>555</v>
       </c>
-      <c r="B41" s="31" t="s">
+      <c r="B41" s="26" t="s">
         <v>556</v>
       </c>
-      <c r="C41" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="30" t="s">
+      <c r="C41" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E41" s="31" t="s">
+      <c r="E41" s="26" t="s">
         <v>557</v>
       </c>
-      <c r="F41" s="31" t="s">
+      <c r="F41" s="26" t="s">
         <v>558</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="28" t="s">
+      <c r="A42" s="23" t="s">
         <v>559</v>
       </c>
-      <c r="B42" s="31" t="s">
+      <c r="B42" s="26" t="s">
         <v>560</v>
       </c>
-      <c r="C42" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D42" s="30" t="s">
+      <c r="C42" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D42" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="E42" s="31" t="s">
+      <c r="E42" s="26" t="s">
         <v>561</v>
       </c>
-      <c r="F42" s="31" t="s">
+      <c r="F42" s="26" t="s">
         <v>562</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="28" t="s">
+      <c r="A43" s="23" t="s">
         <v>563</v>
       </c>
-      <c r="B43" s="31" t="s">
+      <c r="B43" s="26" t="s">
         <v>564</v>
       </c>
-      <c r="C43" s="32" t="s">
+      <c r="C43" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D43" s="33" t="s">
+      <c r="D43" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="E43" s="31" t="s">
+      <c r="E43" s="26" t="s">
         <v>561</v>
       </c>
-      <c r="F43" s="31" t="s">
+      <c r="F43" s="26" t="s">
         <v>565</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="28" t="s">
+      <c r="A44" s="23" t="s">
         <v>566</v>
       </c>
-      <c r="B44" s="31" t="s">
+      <c r="B44" s="26" t="s">
         <v>567</v>
       </c>
-      <c r="C44" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="30" t="s">
+      <c r="C44" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E44" s="31" t="s">
+      <c r="E44" s="26" t="s">
         <v>568</v>
       </c>
-      <c r="F44" s="31" t="s">
+      <c r="F44" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="28" t="s">
+      <c r="A45" s="23" t="s">
         <v>569</v>
       </c>
-      <c r="B45" s="31" t="s">
+      <c r="B45" s="26" t="s">
         <v>570</v>
       </c>
-      <c r="C45" s="32" t="s">
+      <c r="C45" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D45" s="33" t="s">
+      <c r="D45" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="31" t="s">
+      <c r="E45" s="26" t="s">
         <v>571</v>
       </c>
-      <c r="F45" s="31" t="s">
+      <c r="F45" s="26" t="s">
         <v>572</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="28" t="s">
+      <c r="A46" s="23" t="s">
         <v>573</v>
       </c>
-      <c r="B46" s="31" t="s">
+      <c r="B46" s="26" t="s">
         <v>574</v>
       </c>
-      <c r="C46" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="30" t="s">
+      <c r="C46" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E46" s="31" t="s">
+      <c r="E46" s="26" t="s">
         <v>575</v>
       </c>
-      <c r="F46" s="31" t="s">
+      <c r="F46" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="28" t="s">
+      <c r="A47" s="23" t="s">
         <v>576</v>
       </c>
-      <c r="B47" s="31" t="s">
+      <c r="B47" s="26" t="s">
         <v>577</v>
       </c>
-      <c r="C47" s="32" t="s">
+      <c r="C47" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D47" s="33" t="s">
+      <c r="D47" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="31" t="s">
+      <c r="E47" s="26" t="s">
         <v>571</v>
       </c>
-      <c r="F47" s="31" t="s">
+      <c r="F47" s="26" t="s">
         <v>578</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="28" t="s">
+      <c r="A48" s="23" t="s">
         <v>579</v>
       </c>
-      <c r="B48" s="31" t="s">
+      <c r="B48" s="26" t="s">
         <v>580</v>
       </c>
-      <c r="C48" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D48" s="30" t="s">
+      <c r="C48" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="E48" s="31" t="s">
+      <c r="E48" s="26" t="s">
         <v>581</v>
       </c>
-      <c r="F48" s="31" t="s">
+      <c r="F48" s="26" t="s">
         <v>582</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="28" t="s">
+      <c r="A49" s="23" t="s">
         <v>583</v>
       </c>
-      <c r="B49" s="31" t="s">
+      <c r="B49" s="26" t="s">
         <v>584</v>
       </c>
-      <c r="C49" s="32" t="s">
+      <c r="C49" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D49" s="33" t="s">
+      <c r="D49" s="28" t="s">
         <v>114</v>
       </c>
-      <c r="E49" s="31" t="s">
+      <c r="E49" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F49" s="31" t="s">
+      <c r="F49" s="26" t="s">
         <v>585</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="28" t="s">
+      <c r="A50" s="23" t="s">
         <v>586</v>
       </c>
-      <c r="B50" s="31" t="s">
+      <c r="B50" s="26" t="s">
         <v>587</v>
       </c>
-      <c r="C50" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="30" t="s">
+      <c r="C50" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E50" s="31" t="s">
+      <c r="E50" s="26" t="s">
         <v>588</v>
       </c>
-      <c r="F50" s="31" t="s">
+      <c r="F50" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="28" t="s">
+      <c r="A51" s="23" t="s">
         <v>589</v>
       </c>
-      <c r="B51" s="31" t="s">
+      <c r="B51" s="26" t="s">
         <v>590</v>
       </c>
-      <c r="C51" s="32" t="s">
+      <c r="C51" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D51" s="33" t="s">
+      <c r="D51" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="E51" s="31" t="s">
+      <c r="E51" s="26" t="s">
         <v>591</v>
       </c>
-      <c r="F51" s="31" t="s">
+      <c r="F51" s="26" t="s">
         <v>592</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="28" t="s">
+      <c r="A52" s="23" t="s">
         <v>593</v>
       </c>
-      <c r="B52" s="31" t="s">
+      <c r="B52" s="26" t="s">
         <v>594</v>
       </c>
-      <c r="C52" s="32" t="s">
+      <c r="C52" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D52" s="33" t="s">
+      <c r="D52" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E52" s="31" t="s">
+      <c r="E52" s="26" t="s">
         <v>595</v>
       </c>
-      <c r="F52" s="31" t="s">
+      <c r="F52" s="26" t="s">
         <v>596</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="28" t="s">
+      <c r="A53" s="23" t="s">
         <v>597</v>
       </c>
-      <c r="B53" s="31" t="s">
+      <c r="B53" s="26" t="s">
         <v>598</v>
       </c>
-      <c r="C53" s="32" t="s">
+      <c r="C53" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D53" s="33" t="s">
+      <c r="D53" s="28" t="s">
         <v>95</v>
       </c>
-      <c r="E53" s="31" t="s">
+      <c r="E53" s="26" t="s">
         <v>599</v>
       </c>
-      <c r="F53" s="31" t="s">
+      <c r="F53" s="26" t="s">
         <v>600</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="28" t="s">
+      <c r="A54" s="23" t="s">
         <v>601</v>
       </c>
-      <c r="B54" s="31" t="s">
+      <c r="B54" s="26" t="s">
         <v>602</v>
       </c>
-      <c r="C54" s="32" t="s">
+      <c r="C54" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D54" s="33" t="s">
+      <c r="D54" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="E54" s="31" t="s">
+      <c r="E54" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F54" s="31" t="s">
+      <c r="F54" s="26" t="s">
         <v>603</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="28" t="s">
+      <c r="A55" s="23" t="s">
         <v>604</v>
       </c>
-      <c r="B55" s="31" t="s">
+      <c r="B55" s="26" t="s">
         <v>605</v>
       </c>
-      <c r="C55" s="32" t="s">
+      <c r="C55" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D55" s="33" t="s">
+      <c r="D55" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="E55" s="31" t="s">
+      <c r="E55" s="26" t="s">
         <v>606</v>
       </c>
-      <c r="F55" s="31" t="s">
+      <c r="F55" s="26" t="s">
         <v>607</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="28" t="s">
+      <c r="A56" s="23" t="s">
         <v>608</v>
       </c>
-      <c r="B56" s="31" t="s">
+      <c r="B56" s="26" t="s">
         <v>609</v>
       </c>
-      <c r="C56" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" s="30" t="s">
+      <c r="C56" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E56" s="31" t="s">
+      <c r="E56" s="26" t="s">
         <v>610</v>
       </c>
-      <c r="F56" s="31" t="s">
+      <c r="F56" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="28" t="s">
+      <c r="A57" s="23" t="s">
         <v>611</v>
       </c>
-      <c r="B57" s="31" t="s">
+      <c r="B57" s="26" t="s">
         <v>612</v>
       </c>
-      <c r="C57" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D57" s="30" t="s">
+      <c r="C57" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="E57" s="31" t="s">
+      <c r="E57" s="26" t="s">
         <v>610</v>
       </c>
-      <c r="F57" s="31" t="s">
+      <c r="F57" s="26" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="28" t="s">
+      <c r="A58" s="23" t="s">
         <v>613</v>
       </c>
-      <c r="B58" s="31" t="s">
+      <c r="B58" s="26" t="s">
         <v>614</v>
       </c>
-      <c r="C58" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D58" s="30" t="s">
+      <c r="C58" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D58" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E58" s="31" t="s">
+      <c r="E58" s="26" t="s">
         <v>615</v>
       </c>
-      <c r="F58" s="31" t="s">
+      <c r="F58" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="28" t="s">
+      <c r="A59" s="23" t="s">
         <v>616</v>
       </c>
-      <c r="B59" s="31" t="s">
+      <c r="B59" s="26" t="s">
         <v>617</v>
       </c>
-      <c r="C59" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" s="30" t="s">
+      <c r="C59" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D59" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="E59" s="31" t="s">
+      <c r="E59" s="26" t="s">
         <v>615</v>
       </c>
-      <c r="F59" s="31" t="s">
+      <c r="F59" s="26" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A60" s="28" t="s">
+      <c r="A60" s="23" t="s">
         <v>618</v>
       </c>
-      <c r="B60" s="31" t="s">
+      <c r="B60" s="26" t="s">
         <v>619</v>
       </c>
-      <c r="C60" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D60" s="30" t="s">
+      <c r="C60" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D60" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E60" s="31" t="s">
+      <c r="E60" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F60" s="31" t="s">
+      <c r="F60" s="26" t="s">
         <v>620</v>
       </c>
     </row>
@@ -7310,142 +7292,142 @@
       <c r="F61" s="4"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A62" s="28" t="s">
+      <c r="A62" s="23" t="s">
         <v>622</v>
       </c>
-      <c r="B62" s="31" t="s">
+      <c r="B62" s="26" t="s">
         <v>623</v>
       </c>
-      <c r="C62" s="32" t="s">
+      <c r="C62" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D62" s="33" t="s">
+      <c r="D62" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="E62" s="31" t="s">
+      <c r="E62" s="26" t="s">
         <v>624</v>
       </c>
-      <c r="F62" s="31" t="s">
+      <c r="F62" s="26" t="s">
         <v>625</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A63" s="28" t="s">
+      <c r="A63" s="23" t="s">
         <v>626</v>
       </c>
-      <c r="B63" s="31" t="s">
+      <c r="B63" s="26" t="s">
         <v>627</v>
       </c>
-      <c r="C63" s="32" t="s">
+      <c r="C63" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D63" s="33" t="s">
+      <c r="D63" s="28" t="s">
         <v>230</v>
       </c>
-      <c r="E63" s="31" t="s">
+      <c r="E63" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F63" s="31" t="s">
+      <c r="F63" s="26" t="s">
         <v>628</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A64" s="28" t="s">
+      <c r="A64" s="23" t="s">
         <v>629</v>
       </c>
-      <c r="B64" s="31" t="s">
+      <c r="B64" s="26" t="s">
         <v>630</v>
       </c>
-      <c r="C64" s="32" t="s">
+      <c r="C64" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D64" s="33" t="s">
+      <c r="D64" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="E64" s="31" t="s">
+      <c r="E64" s="26" t="s">
         <v>631</v>
       </c>
-      <c r="F64" s="31" t="s">
+      <c r="F64" s="26" t="s">
         <v>632</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A65" s="28" t="s">
+      <c r="A65" s="23" t="s">
         <v>633</v>
       </c>
-      <c r="B65" s="31" t="s">
+      <c r="B65" s="26" t="s">
         <v>634</v>
       </c>
-      <c r="C65" s="32" t="s">
+      <c r="C65" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="D65" s="33" t="s">
+      <c r="D65" s="28" t="s">
         <v>230</v>
       </c>
-      <c r="E65" s="31" t="s">
+      <c r="E65" s="26" t="s">
         <v>635</v>
       </c>
-      <c r="F65" s="31" t="s">
+      <c r="F65" s="26" t="s">
         <v>636</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A66" s="28" t="s">
+      <c r="A66" s="23" t="s">
         <v>637</v>
       </c>
-      <c r="B66" s="31" t="s">
+      <c r="B66" s="26" t="s">
         <v>638</v>
       </c>
-      <c r="C66" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="30" t="s">
+      <c r="C66" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="E66" s="31" t="s">
+      <c r="E66" s="26" t="s">
         <v>501</v>
       </c>
-      <c r="F66" s="31" t="s">
+      <c r="F66" s="26" t="s">
         <v>639</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A67" s="28" t="s">
+      <c r="A67" s="23" t="s">
         <v>640</v>
       </c>
-      <c r="B67" s="31" t="s">
+      <c r="B67" s="26" t="s">
         <v>641</v>
       </c>
-      <c r="C67" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D67" s="30" t="s">
+      <c r="C67" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E67" s="31" t="s">
+      <c r="E67" s="26" t="s">
         <v>642</v>
       </c>
-      <c r="F67" s="31" t="s">
+      <c r="F67" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A68" s="28" t="s">
+      <c r="A68" s="23" t="s">
         <v>643</v>
       </c>
-      <c r="B68" s="31" t="s">
+      <c r="B68" s="26" t="s">
         <v>644</v>
       </c>
-      <c r="C68" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D68" s="30" t="s">
+      <c r="C68" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D68" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E68" s="31" t="s">
+      <c r="E68" s="26" t="s">
         <v>645</v>
       </c>
-      <c r="F68" s="31" t="s">
+      <c r="F68" s="26" t="s">
         <v>482</v>
       </c>
     </row>
@@ -7460,242 +7442,242 @@
       <c r="F69" s="4"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A70" s="28" t="s">
+      <c r="A70" s="23" t="s">
         <v>647</v>
       </c>
-      <c r="B70" s="31" t="s">
+      <c r="B70" s="26" t="s">
         <v>648</v>
       </c>
-      <c r="C70" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="30" t="s">
+      <c r="C70" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E70" s="31" t="s">
+      <c r="E70" s="26" t="s">
         <v>649</v>
       </c>
-      <c r="F70" s="31" t="s">
+      <c r="F70" s="26" t="s">
         <v>650</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A71" s="28" t="s">
+      <c r="A71" s="23" t="s">
         <v>651</v>
       </c>
-      <c r="B71" s="31" t="s">
+      <c r="B71" s="26" t="s">
         <v>652</v>
       </c>
-      <c r="C71" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="30" t="s">
+      <c r="C71" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D71" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E71" s="31" t="s">
+      <c r="E71" s="26" t="s">
         <v>649</v>
       </c>
-      <c r="F71" s="31" t="s">
+      <c r="F71" s="26" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A72" s="28" t="s">
+      <c r="A72" s="23" t="s">
         <v>654</v>
       </c>
-      <c r="B72" s="31" t="s">
+      <c r="B72" s="26" t="s">
         <v>655</v>
       </c>
-      <c r="C72" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72" s="30" t="s">
+      <c r="C72" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E72" s="31" t="s">
+      <c r="E72" s="26" t="s">
         <v>656</v>
       </c>
-      <c r="F72" s="31" t="s">
+      <c r="F72" s="26" t="s">
         <v>657</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="28" t="s">
+      <c r="A73" s="23" t="s">
         <v>658</v>
       </c>
-      <c r="B73" s="31" t="s">
+      <c r="B73" s="26" t="s">
         <v>659</v>
       </c>
-      <c r="C73" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D73" s="30" t="s">
+      <c r="C73" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E73" s="31" t="s">
+      <c r="E73" s="26" t="s">
         <v>656</v>
       </c>
-      <c r="F73" s="31" t="s">
+      <c r="F73" s="26" t="s">
         <v>660</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="28" t="s">
+      <c r="A74" s="23" t="s">
         <v>661</v>
       </c>
-      <c r="B74" s="31" t="s">
+      <c r="B74" s="26" t="s">
         <v>662</v>
       </c>
-      <c r="C74" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D74" s="30" t="s">
+      <c r="C74" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E74" s="31" t="s">
+      <c r="E74" s="26" t="s">
         <v>663</v>
       </c>
-      <c r="F74" s="31" t="s">
+      <c r="F74" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="28" t="s">
+      <c r="A75" s="23" t="s">
         <v>664</v>
       </c>
-      <c r="B75" s="31" t="s">
+      <c r="B75" s="26" t="s">
         <v>665</v>
       </c>
-      <c r="C75" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D75" s="30" t="s">
+      <c r="C75" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D75" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E75" s="31" t="s">
+      <c r="E75" s="26" t="s">
         <v>663</v>
       </c>
-      <c r="F75" s="31" t="s">
+      <c r="F75" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A76" s="28" t="s">
+      <c r="A76" s="23" t="s">
         <v>666</v>
       </c>
-      <c r="B76" s="31" t="s">
+      <c r="B76" s="26" t="s">
         <v>667</v>
       </c>
-      <c r="C76" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D76" s="30" t="s">
+      <c r="C76" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E76" s="31" t="s">
+      <c r="E76" s="26" t="s">
         <v>663</v>
       </c>
-      <c r="F76" s="31" t="s">
+      <c r="F76" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A77" s="28" t="s">
+      <c r="A77" s="23" t="s">
         <v>668</v>
       </c>
-      <c r="B77" s="31" t="s">
+      <c r="B77" s="26" t="s">
         <v>669</v>
       </c>
-      <c r="C77" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D77" s="30" t="s">
+      <c r="C77" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D77" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E77" s="31" t="s">
+      <c r="E77" s="26" t="s">
         <v>670</v>
       </c>
-      <c r="F77" s="31" t="s">
+      <c r="F77" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A78" s="28" t="s">
+      <c r="A78" s="23" t="s">
         <v>671</v>
       </c>
-      <c r="B78" s="31" t="s">
+      <c r="B78" s="26" t="s">
         <v>672</v>
       </c>
-      <c r="C78" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D78" s="30" t="s">
+      <c r="C78" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D78" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E78" s="31" t="s">
+      <c r="E78" s="26" t="s">
         <v>670</v>
       </c>
-      <c r="F78" s="31" t="s">
+      <c r="F78" s="26" t="s">
         <v>482</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A79" s="28" t="s">
+      <c r="A79" s="23" t="s">
         <v>673</v>
       </c>
-      <c r="B79" s="31" t="s">
+      <c r="B79" s="26" t="s">
         <v>674</v>
       </c>
-      <c r="C79" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D79" s="30" t="s">
+      <c r="C79" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D79" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E79" s="31" t="s">
+      <c r="E79" s="26" t="s">
         <v>670</v>
       </c>
-      <c r="F79" s="31" t="s">
+      <c r="F79" s="26" t="s">
         <v>675</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A80" s="28" t="s">
+      <c r="A80" s="23" t="s">
         <v>676</v>
       </c>
-      <c r="B80" s="31" t="s">
+      <c r="B80" s="26" t="s">
         <v>677</v>
       </c>
-      <c r="C80" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D80" s="30" t="s">
+      <c r="C80" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D80" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E80" s="31" t="s">
+      <c r="E80" s="26" t="s">
         <v>678</v>
       </c>
-      <c r="F80" s="31" t="s">
+      <c r="F80" s="26" t="s">
         <v>679</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A81" s="28" t="s">
+      <c r="A81" s="23" t="s">
         <v>680</v>
       </c>
-      <c r="B81" s="31" t="s">
+      <c r="B81" s="26" t="s">
         <v>681</v>
       </c>
-      <c r="C81" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="D81" s="30" t="s">
+      <c r="C81" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D81" s="25" t="s">
         <v>451</v>
       </c>
-      <c r="E81" s="31" t="s">
+      <c r="E81" s="26" t="s">
         <v>682</v>
       </c>
-      <c r="F81" s="31" t="s">
+      <c r="F81" s="26" t="s">
         <v>683</v>
       </c>
     </row>
@@ -7711,10 +7693,10 @@
       <c r="B84" s="1" t="s">
         <v>686</v>
       </c>
-      <c r="C84" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D84" s="34" t="s">
+      <c r="C84" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D84" s="31" t="s">
         <v>85</v>
       </c>
       <c r="E84" s="1" t="s">
@@ -7731,10 +7713,10 @@
       <c r="B85" s="1" t="s">
         <v>689</v>
       </c>
-      <c r="C85" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D85" s="34" t="s">
+      <c r="C85" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" s="31" t="s">
         <v>18</v>
       </c>
       <c r="E85" s="1" t="s">
@@ -7751,10 +7733,10 @@
       <c r="B86" s="1" t="s">
         <v>692</v>
       </c>
-      <c r="C86" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D86" s="34" t="s">
+      <c r="C86" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D86" s="31" t="s">
         <v>18</v>
       </c>
       <c r="E86" s="1" t="s">
@@ -7771,10 +7753,10 @@
       <c r="B87" s="1" t="s">
         <v>695</v>
       </c>
-      <c r="C87" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D87" s="34" t="s">
+      <c r="C87" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D87" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E87" s="1" t="s">
@@ -7791,10 +7773,10 @@
       <c r="B88" s="1" t="s">
         <v>699</v>
       </c>
-      <c r="C88" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D88" s="34" t="s">
+      <c r="C88" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E88" s="1" t="s">
@@ -7811,10 +7793,10 @@
       <c r="B89" s="1" t="s">
         <v>702</v>
       </c>
-      <c r="C89" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D89" s="34" t="s">
+      <c r="C89" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" s="31" t="s">
         <v>18</v>
       </c>
       <c r="E89" s="1" t="s">
@@ -7831,10 +7813,10 @@
       <c r="B90" s="1" t="s">
         <v>705</v>
       </c>
-      <c r="C90" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D90" s="34" t="s">
+      <c r="C90" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D90" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E90" s="1" t="s">
@@ -7851,10 +7833,10 @@
       <c r="B91" s="1" t="s">
         <v>709</v>
       </c>
-      <c r="C91" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D91" s="34" t="s">
+      <c r="C91" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D91" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E91" s="1" t="s">
@@ -7871,10 +7853,10 @@
       <c r="B92" s="1" t="s">
         <v>712</v>
       </c>
-      <c r="C92" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D92" s="34" t="s">
+      <c r="C92" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D92" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E92" s="1" t="s">
@@ -7891,10 +7873,10 @@
       <c r="B93" s="1" t="s">
         <v>716</v>
       </c>
-      <c r="C93" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="D93" s="34" t="s">
+      <c r="C93" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" s="31" t="s">
         <v>47</v>
       </c>
       <c r="E93" s="1" t="s">
@@ -7985,242 +7967,242 @@
       <c r="F4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="23" t="s">
         <v>723</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="26" t="s">
         <v>724</v>
       </c>
-      <c r="C5" s="31" t="s">
+      <c r="C5" s="26" t="s">
         <v>725</v>
       </c>
-      <c r="D5" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="29" t="s">
+      <c r="D5" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="26" t="s">
         <v>726</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="23" t="s">
         <v>727</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="26" t="s">
         <v>728</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="26" t="s">
         <v>729</v>
       </c>
-      <c r="D6" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="29" t="s">
+      <c r="D6" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="26" t="s">
         <v>730</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="23" t="s">
         <v>731</v>
       </c>
-      <c r="B7" s="31" t="s">
+      <c r="B7" s="26" t="s">
         <v>732</v>
       </c>
-      <c r="C7" s="31" t="s">
+      <c r="C7" s="26" t="s">
         <v>733</v>
       </c>
-      <c r="D7" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="29" t="s">
+      <c r="D7" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="26" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="23" t="s">
         <v>734</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="26" t="s">
         <v>735</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="26" t="s">
         <v>736</v>
       </c>
-      <c r="D8" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="29" t="s">
+      <c r="D8" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="26" t="s">
         <v>737</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="23" t="s">
         <v>738</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="26" t="s">
         <v>739</v>
       </c>
-      <c r="C9" s="31" t="s">
+      <c r="C9" s="26" t="s">
         <v>740</v>
       </c>
-      <c r="D9" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="29" t="s">
+      <c r="D9" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="26" t="s">
         <v>741</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="23" t="s">
         <v>742</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="26" t="s">
         <v>743</v>
       </c>
-      <c r="C10" s="31" t="s">
+      <c r="C10" s="26" t="s">
         <v>744</v>
       </c>
-      <c r="D10" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" s="29" t="s">
+      <c r="D10" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="26" t="s">
         <v>745</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="23" t="s">
         <v>746</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="26" t="s">
         <v>747</v>
       </c>
-      <c r="C11" s="31" t="s">
+      <c r="C11" s="26" t="s">
         <v>748</v>
       </c>
-      <c r="D11" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="29" t="s">
+      <c r="D11" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="26" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="23" t="s">
         <v>750</v>
       </c>
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="26" t="s">
         <v>751</v>
       </c>
-      <c r="C12" s="31" t="s">
+      <c r="C12" s="26" t="s">
         <v>752</v>
       </c>
-      <c r="D12" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="29" t="s">
+      <c r="D12" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="26" t="s">
         <v>753</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="23" t="s">
         <v>754</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="26" t="s">
         <v>755</v>
       </c>
-      <c r="C13" s="31" t="s">
+      <c r="C13" s="26" t="s">
         <v>756</v>
       </c>
-      <c r="D13" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="29" t="s">
+      <c r="D13" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="26" t="s">
         <v>757</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>758</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="26" t="s">
         <v>759</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="26" t="s">
         <v>760</v>
       </c>
-      <c r="D14" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="29" t="s">
+      <c r="D14" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="26" t="s">
         <v>761</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
+      <c r="A15" s="23" t="s">
         <v>762</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="26" t="s">
         <v>763</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="26" t="s">
         <v>764</v>
       </c>
-      <c r="D15" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="29" t="s">
+      <c r="D15" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="24" t="s">
         <v>200</v>
       </c>
-      <c r="F15" s="31" t="s">
+      <c r="F15" s="26" t="s">
         <v>765</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="23" t="s">
         <v>766</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="26" t="s">
         <v>767</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="C16" s="26" t="s">
         <v>768</v>
       </c>
-      <c r="D16" s="32" t="s">
+      <c r="D16" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="32" t="s">
+      <c r="E16" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="F16" s="31" t="s">
+      <c r="F16" s="26" t="s">
         <v>769</v>
       </c>
     </row>
@@ -8235,182 +8217,182 @@
       <c r="F17" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="23" t="s">
         <v>771</v>
       </c>
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="26" t="s">
         <v>772</v>
       </c>
-      <c r="C18" s="31" t="s">
+      <c r="C18" s="26" t="s">
         <v>773</v>
       </c>
-      <c r="D18" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="29" t="s">
+      <c r="D18" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="31" t="s">
+      <c r="F18" s="26" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="A19" s="23" t="s">
         <v>775</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="26" t="s">
         <v>776</v>
       </c>
-      <c r="C19" s="31" t="s">
+      <c r="C19" s="26" t="s">
         <v>777</v>
       </c>
-      <c r="D19" s="32" t="s">
+      <c r="D19" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E19" s="32" t="s">
+      <c r="E19" s="27" t="s">
         <v>230</v>
       </c>
-      <c r="F19" s="31" t="s">
+      <c r="F19" s="26" t="s">
         <v>778</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="28" t="s">
+      <c r="A20" s="23" t="s">
         <v>779</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="26" t="s">
         <v>780</v>
       </c>
-      <c r="C20" s="31" t="s">
+      <c r="C20" s="26" t="s">
         <v>781</v>
       </c>
-      <c r="D20" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="29" t="s">
+      <c r="D20" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F20" s="31" t="s">
+      <c r="F20" s="26" t="s">
         <v>782</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="28" t="s">
+      <c r="A21" s="23" t="s">
         <v>783</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="26" t="s">
         <v>784</v>
       </c>
-      <c r="C21" s="31" t="s">
+      <c r="C21" s="26" t="s">
         <v>785</v>
       </c>
-      <c r="D21" s="32" t="s">
+      <c r="D21" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E21" s="32" t="s">
+      <c r="E21" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="F21" s="31" t="s">
+      <c r="F21" s="26" t="s">
         <v>786</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="28" t="s">
+      <c r="A22" s="23" t="s">
         <v>787</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="26" t="s">
         <v>788</v>
       </c>
-      <c r="C22" s="31" t="s">
+      <c r="C22" s="26" t="s">
         <v>789</v>
       </c>
-      <c r="D22" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E22" s="29" t="s">
+      <c r="D22" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="31" t="s">
+      <c r="F22" s="26" t="s">
         <v>790</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
+      <c r="A23" s="23" t="s">
         <v>791</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="26" t="s">
         <v>792</v>
       </c>
-      <c r="C23" s="31" t="s">
+      <c r="C23" s="26" t="s">
         <v>793</v>
       </c>
-      <c r="D23" s="32" t="s">
+      <c r="D23" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E23" s="32" t="s">
+      <c r="E23" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="F23" s="31" t="s">
+      <c r="F23" s="26" t="s">
         <v>794</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="23" t="s">
         <v>795</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="26" t="s">
         <v>796</v>
       </c>
-      <c r="C24" s="31" t="s">
+      <c r="C24" s="26" t="s">
         <v>797</v>
       </c>
-      <c r="D24" s="32" t="s">
+      <c r="D24" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E24" s="32" t="s">
+      <c r="E24" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="F24" s="31" t="s">
+      <c r="F24" s="26" t="s">
         <v>798</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>799</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="26" t="s">
         <v>800</v>
       </c>
-      <c r="C25" s="31" t="s">
+      <c r="C25" s="26" t="s">
         <v>801</v>
       </c>
-      <c r="D25" s="32" t="s">
+      <c r="D25" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="E25" s="32" t="s">
+      <c r="E25" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="31" t="s">
+      <c r="F25" s="26" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="23" t="s">
         <v>803</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="26" t="s">
         <v>804</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="26" t="s">
         <v>805</v>
       </c>
-      <c r="D26" s="29" t="s">
-        <v>11</v>
-      </c>
-      <c r="E26" s="29" t="s">
+      <c r="D26" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="F26" s="31" t="s">
+      <c r="F26" s="26" t="s">
         <v>369</v>
       </c>
     </row>
@@ -8429,10 +8411,10 @@
       <c r="C29" s="1" t="s">
         <v>809</v>
       </c>
-      <c r="D29" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E29" s="34" t="s">
+      <c r="D29" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="31" t="s">
         <v>47</v>
       </c>
       <c r="F29" s="1" t="s">
@@ -8449,10 +8431,10 @@
       <c r="C30" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="D30" s="34" t="s">
-        <v>11</v>
-      </c>
-      <c r="E30" s="34" t="s">
+      <c r="D30" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="31" t="s">
         <v>200</v>
       </c>
       <c r="F30" s="1" t="s">
@@ -8469,10 +8451,10 @@
       <c r="C31" s="1" t="s">
         <v>817</v>
       </c>
-      <c r="D31" s="35" t="s">
+      <c r="D31" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="E31" s="35" t="s">
+      <c r="E31" s="32" t="s">
         <v>114</v>
       </c>
       <c r="F31" s="1" t="s">
@@ -8489,10 +8471,10 @@
       <c r="C32" s="1" t="s">
         <v>821</v>
       </c>
-      <c r="D32" s="35" t="s">
+      <c r="D32" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="E32" s="35" t="s">
+      <c r="E32" s="32" t="s">
         <v>100</v>
       </c>
       <c r="F32" s="1" t="s">
@@ -8565,342 +8547,342 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="23" t="s">
         <v>827</v>
       </c>
-      <c r="B4" s="36" t="n">
+      <c r="B4" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="C4" s="30" t="n">
+      <c r="C4" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="D4" s="33" t="n">
+      <c r="D4" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="25" t="n">
+      <c r="E4" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="31" t="s">
+      <c r="F4" s="26" t="s">
         <v>828</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="23" t="s">
         <v>829</v>
       </c>
-      <c r="B5" s="36" t="n">
+      <c r="B5" s="33" t="n">
         <v>5</v>
       </c>
-      <c r="C5" s="30" t="n">
+      <c r="C5" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="33" t="n">
+      <c r="D5" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="26" t="s">
         <v>830</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="23" t="s">
         <v>831</v>
       </c>
-      <c r="B6" s="36" t="n">
+      <c r="B6" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="30" t="n">
+      <c r="C6" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="33" t="n">
+      <c r="D6" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="31" t="s">
+      <c r="F6" s="26" t="s">
         <v>832</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="A7" s="23" t="s">
         <v>833</v>
       </c>
-      <c r="B7" s="36" t="n">
+      <c r="B7" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="30" t="n">
+      <c r="C7" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="33" t="n">
+      <c r="D7" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="31" t="s">
+      <c r="F7" s="26" t="s">
         <v>834</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="23" t="s">
         <v>835</v>
       </c>
-      <c r="B8" s="36" t="n">
+      <c r="B8" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="30" t="n">
+      <c r="C8" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="D8" s="33" t="n">
+      <c r="D8" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="26" t="s">
         <v>836</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="23" t="s">
         <v>837</v>
       </c>
-      <c r="B9" s="36" t="n">
+      <c r="B9" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="30" t="n">
+      <c r="C9" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="33" t="n">
+      <c r="D9" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="31" t="s">
+      <c r="F9" s="26" t="s">
         <v>838</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="23" t="s">
         <v>839</v>
       </c>
-      <c r="B10" s="36" t="n">
+      <c r="B10" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="30" t="n">
+      <c r="C10" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="33" t="n">
+      <c r="D10" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="31" t="s">
+      <c r="F10" s="26" t="s">
         <v>840</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="28" t="s">
+      <c r="A11" s="23" t="s">
         <v>841</v>
       </c>
-      <c r="B11" s="36" t="n">
+      <c r="B11" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="C11" s="30" t="n">
+      <c r="C11" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="33" t="n">
+      <c r="D11" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="26" t="s">
         <v>842</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
+      <c r="A12" s="23" t="s">
         <v>843</v>
       </c>
-      <c r="B12" s="36" t="n">
+      <c r="B12" s="33" t="n">
         <v>7</v>
       </c>
-      <c r="C12" s="30" t="n">
+      <c r="C12" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="33" t="n">
+      <c r="D12" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="31" t="s">
+      <c r="F12" s="26" t="s">
         <v>844</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+      <c r="A13" s="23" t="s">
         <v>845</v>
       </c>
-      <c r="B13" s="36" t="n">
+      <c r="B13" s="33" t="n">
         <v>14</v>
       </c>
-      <c r="C13" s="30" t="n">
+      <c r="C13" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="33" t="n">
+      <c r="D13" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="26" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="23" t="s">
         <v>847</v>
       </c>
-      <c r="B14" s="36" t="n">
+      <c r="B14" s="33" t="n">
         <v>9</v>
       </c>
-      <c r="C14" s="30" t="n">
+      <c r="C14" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="33" t="n">
+      <c r="D14" s="28" t="n">
         <v>5</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="31" t="s">
+      <c r="F14" s="26" t="s">
         <v>848</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="23" t="s">
         <v>849</v>
       </c>
-      <c r="B16" s="37" t="n">
+      <c r="B16" s="34" t="n">
         <v>73</v>
       </c>
-      <c r="C16" s="30" t="n">
+      <c r="C16" s="25" t="n">
         <v>33</v>
       </c>
-      <c r="D16" s="33" t="n">
+      <c r="D16" s="28" t="n">
         <v>31</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="F16" s="31"/>
+      <c r="F16" s="26"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38" t="s">
+      <c r="A18" s="35" t="s">
         <v>850</v>
       </c>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="38"/>
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="39" t="s">
+      <c r="A20" s="36" t="s">
         <v>851</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="37" t="s">
         <v>852</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="41" t="s">
+      <c r="A23" s="38" t="s">
         <v>853</v>
       </c>
-      <c r="B23" s="41"/>
-      <c r="C23" s="41"/>
-      <c r="D23" s="41"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="28" t="s">
+      <c r="A24" s="23" t="s">
         <v>854</v>
       </c>
-      <c r="B24" s="31" t="s">
+      <c r="B24" s="26" t="s">
         <v>855</v>
       </c>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="26"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="28" t="s">
+      <c r="A25" s="23" t="s">
         <v>856</v>
       </c>
-      <c r="B25" s="31" t="s">
+      <c r="B25" s="26" t="s">
         <v>857</v>
       </c>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="26"/>
+      <c r="F25" s="26"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="23" t="s">
         <v>858</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="26" t="s">
         <v>859</v>
       </c>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="23" t="s">
         <v>860</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="26" t="s">
         <v>861</v>
       </c>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="31"/>
+      <c r="C27" s="26"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="23" t="s">
         <v>862</v>
       </c>
-      <c r="B28" s="31" t="s">
+      <c r="B28" s="26" t="s">
         <v>863</v>
       </c>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>